<commit_message>
Completa a pasta de artigos com Felten (2021) e Ahn e Carollo (2026)
- felten2021.pdf: versão de trabalho do SSRN da fonte do AIOE, última pendência
  da pasta. A paginação difere da publicada no SMJ, que é a citada no texto.
- ahn2026.pdf: Ahn e Carollo, fluxos do mercado de trabalho americano por
  exposição e adoção de inteligência artificial, versão preliminar de 16 de
  setembro de 2026. Ainda não citado.
- Planilha regenerada: 18 obras, 17 com PDF. Só a base de microdados fica sem
  arquivo, por não ter PDF.
- scripts/bibliografia.py registra as duas obras novas e conta como PDF apenas
  as linhas que apontam para um arquivo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/artigos/referencias_citadas.xlsx
+++ b/artigos/referencias_citadas.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Referências citadas" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Referências citadas'!$A$1:$P$18</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Referências citadas'!$A$1:$P$19</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="219">
   <si>
     <t xml:space="preserve">Chave</t>
   </si>
@@ -352,10 +352,13 @@
     <t xml:space="preserve">Fonte do AIOE, o tratamento principal do trabalho.</t>
   </si>
   <si>
-    <t xml:space="preserve">falta baixar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restrito (SMJ); baixar por acesso institucional do IDP</t>
+    <t xml:space="preserve">felten2021.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Versão de trabalho do SSRN; publicado no SMJ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aberto no SSRN (versão de trabalho); publicado restrito no SMJ</t>
   </si>
   <si>
     <t xml:space="preserve">higano2023</t>
@@ -635,6 +638,36 @@
   </si>
   <si>
     <t xml:space="preserve">Aberto (site, sem PDF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ahn2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ahn, Hie Joo; Carollo, Nicholas A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Artificial intelligence and labor market reallocation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Board of Governors of the Federal Reserve System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ncarollo.net/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ainda não citado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fluxos do mercado de trabalho por exposição e adoção; margem de ajuste no lado da contratação. Inclusão em avaliação.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ahn2026.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Versão preliminar de 16 set. 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aberto (página do autor e site de conferência do NBER)</t>
   </si>
   <si>
     <t xml:space="preserve">Total de obras</t>
@@ -1068,7 +1101,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -1520,39 +1553,41 @@
       <c r="N9" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="O9" s="2"/>
+      <c r="O9" s="2" t="s">
+        <v>110</v>
+      </c>
       <c r="P9" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>2023</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
         <v>20</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>1</v>
@@ -1561,33 +1596,33 @@
         <v>25</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>45</v>
@@ -1596,11 +1631,11 @@
         <v>68</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>4</v>
@@ -1609,44 +1644,44 @@
         <v>37</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>45</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>1</v>
@@ -1655,46 +1690,46 @@
         <v>25</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>2015</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
         <v>20</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>1</v>
@@ -1703,13 +1738,13 @@
         <v>25</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="P13" s="2" t="s">
         <v>41</v>
@@ -1717,30 +1752,30 @@
     </row>
     <row r="14" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C14" s="2" t="n">
         <v>2022</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>1</v>
@@ -1749,61 +1784,61 @@
         <v>25</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>2023</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
         <v>20</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="P15" s="2" t="s">
         <v>41</v>
@@ -1811,34 +1846,34 @@
     </row>
     <row r="16" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>2020</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>20</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>1</v>
@@ -1847,13 +1882,13 @@
         <v>25</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="P16" s="2" t="s">
         <v>41</v>
@@ -1861,30 +1896,30 @@
     </row>
     <row r="17" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>2024</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K17" s="2" t="n">
         <v>1</v>
@@ -1893,42 +1928,42 @@
         <v>25</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C18" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="K18" s="2" t="n">
         <v>1</v>
@@ -1937,50 +1972,94 @@
         <v>83</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" s="2" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="B20" s="4" t="n">
-        <f aca="false">COUNTA(A2:A18)</f>
-        <v>17</v>
+    </row>
+    <row r="19" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="O19" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="B21" s="4" t="n">
-        <f aca="false">SUM(K2:K18)</f>
-        <v>41</v>
+        <f aca="false">COUNTA(A2:A19)</f>
+        <v>18</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="B22" s="4" t="n">
-        <f aca="false">COUNTIF(N2:N18,"&lt;&gt;falta baixar")</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
-        <v>207</v>
+        <f aca="false">SUM(K2:K19)</f>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="B23" s="4" t="n">
+        <f aca="false">COUNTIF(N2:N19,"*.pdf")</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P18"/>
+  <autoFilter ref="A1:P19"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Adiciona Yin, Vu e Persico (2026) à pasta de artigos
Estudo de replicação com vários modelos que mostra instabilidade das medidas de
exposição ocupacional geradas por modelos de linguagem: a exposição média diverge
até 3,6 vezes entre modelos e os coeficientes de diferenças em diferenças variam
2,4 vezes conforme o anotador. Sustenta a ressalva sobre a medida de tratamento e
a previsão de usar mais de uma medida. Ainda não citado.

O README registra também o Felten, Raj e Seamans de 2023, sobre exposição
específica a inteligência artificial generativa, que o SSRN não permite baixar
automaticamente.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/artigos/referencias_citadas.xlsx
+++ b/artigos/referencias_citadas.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Referências citadas" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Referências citadas'!$A$1:$P$19</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Referências citadas'!$A$1:$P$20</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="229">
   <si>
     <t xml:space="preserve">Chave</t>
   </si>
@@ -640,6 +640,39 @@
     <t xml:space="preserve">Aberto (site, sem PDF)</t>
   </si>
   <si>
+    <t xml:space="preserve">yin2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yin, Michelle; Vu, Hoa; Persico, Claudia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How (un)stable are LLM occupational exposure scores?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">evidence from multi-model replication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n. 35110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nber.org/papers/w35110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ainda não citado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instabilidade das medidas de exposição geradas por modelos de linguagem; sustenta a ressalva sobre a medida de tratamento. Inclusão em avaliação.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yin2026.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NBER WP 35110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aberto (NBER); também em pré-print no SSRN</t>
+  </si>
+  <si>
     <t xml:space="preserve">ahn2026</t>
   </si>
   <si>
@@ -653,9 +686,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.ncarollo.net/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ainda não citado</t>
   </si>
   <si>
     <t xml:space="preserve">Fluxos do mercado de trabalho por exposição e adoção; margem de ajuste no lado da contratação. Inclusão em avaliação.</t>
@@ -1101,7 +1131,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -1995,71 +2025,119 @@
       <c r="D19" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="E19" s="2"/>
+      <c r="E19" s="2" t="s">
+        <v>208</v>
+      </c>
       <c r="F19" s="2" t="s">
         <v>45</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="H19" s="2"/>
+        <v>68</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>209</v>
+      </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="M19" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="O19" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="N19" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="O19" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="P19" s="2" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="B21" s="4" t="n">
-        <f aca="false">COUNTA(A2:A19)</f>
-        <v>18</v>
+      <c r="M20" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="N20" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="O20" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="P20" s="2" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="B22" s="4" t="n">
-        <f aca="false">SUM(K2:K19)</f>
-        <v>41</v>
+        <f aca="false">COUNTA(A2:A20)</f>
+        <v>19</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="B23" s="4" t="n">
-        <f aca="false">COUNTIF(N2:N19,"*.pdf")</f>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="s">
-        <v>218</v>
+        <f aca="false">SUM(K2:K20)</f>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B24" s="4" t="n">
+        <f aca="false">COUNTIF(N2:N20,"*.pdf")</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P19"/>
+  <autoFilter ref="A1:P20"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Acrescenta a dimensão de especialização de Autor e Thompson (2025)
- Seção 2.2: ao quadro de tarefas soma-se a segunda dimensão do artigo, em que o
  efeito depende de a remoção de tarefas elevar ou reduzir a especialização
  exigida pelas remanescentes, com sinais opostos entre rendimento e emprego.
  Registra a consequência para o desenho: um índice único por ocupação não
  distingue os dois casos.
- Capítulo 4: o sinal negativo nas margens de vínculo passa a ser lido como
  compatível com o ramo em que o ajuste recai sobre o rendimento, deixando claro
  que compatibilidade não é teste e que a margem de preço não é observada.
- artigos/autor2025.pdf, entrada no referencias.bib pela versão da JEEA e
  planilha regenerada: 20 obras, 19 com PDF.
- dissertacao/versoes: cópia datada do PDF desta etapa.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/artigos/referencias_citadas.xlsx
+++ b/artigos/referencias_citadas.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Referências citadas" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Referências citadas'!$A$1:$P$20</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Referências citadas'!$A$1:$P$21</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="241">
   <si>
     <t xml:space="preserve">Chave</t>
   </si>
@@ -149,6 +149,42 @@
   </si>
   <si>
     <t xml:space="preserve">Restrito (periódico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">autor2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autor, David; Thompson, Neil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expertise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Journal of the European Economic Association</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v. 23, n. 4, p. 1203-1271</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1093/jeea/jvaf023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1093/jeea/jvaf023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cap. 2 Referencial; Cap. 4 Resultados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimensão de especialização das tarefas remanescentes; sinais opostos entre rendimento e emprego.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">autor2025.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NBER WP 33941; publicado na JEEA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restrito na JEEA; versão aberta no NBER e na página do MIT</t>
   </si>
   <si>
     <t xml:space="preserve">ibge2022tratamento</t>
@@ -1131,7 +1167,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -1302,7 +1338,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>42</v>
       </c>
@@ -1310,22 +1346,24 @@
         <v>43</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>44</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
         <v>48</v>
       </c>
@@ -1348,7 +1386,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>54</v>
       </c>
@@ -1356,123 +1394,121 @@
         <v>55</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>56</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2" t="s">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="I5" s="2" t="s">
         <v>59</v>
       </c>
+      <c r="I5" s="2"/>
       <c r="J5" s="2" t="s">
         <v>60</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="I6" s="2"/>
+        <v>70</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="J6" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>71</v>
+        <v>37</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2" t="s">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="I7" s="2" t="s">
         <v>81</v>
       </c>
+      <c r="I7" s="2"/>
       <c r="J7" s="2" t="s">
         <v>82</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>83</v>
@@ -1487,25 +1523,23 @@
         <v>86</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>41</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="E8" s="2" t="s">
         <v>90</v>
       </c>
+      <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
         <v>20</v>
       </c>
@@ -1522,22 +1556,22 @@
         <v>94</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>37</v>
+        <v>95</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>98</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1548,7 +1582,7 @@
         <v>100</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>101</v>
@@ -1572,38 +1606,40 @@
         <v>106</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L9" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M9" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="N9" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="O9" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="O9" s="2" t="s">
+      <c r="P9" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="P9" s="2" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C10" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
         <v>20</v>
       </c>
@@ -1620,146 +1656,146 @@
         <v>118</v>
       </c>
       <c r="K10" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="K11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="M10" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="O10" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="P10" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="K11" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="M11" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="H12" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>139</v>
+      </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>2015</v>
+        <v>2026</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="E13" s="2"/>
+        <v>147</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>148</v>
+      </c>
       <c r="F13" s="2" t="s">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>148</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
       <c r="J13" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>1</v>
@@ -1768,44 +1804,46 @@
         <v>25</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>41</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2022</v>
+        <v>2015</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="I14" s="2"/>
+        <v>159</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>160</v>
+      </c>
       <c r="J14" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>1</v>
@@ -1814,52 +1852,50 @@
         <v>25</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>162</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
         <v>20</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>168</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="I15" s="2"/>
       <c r="J15" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>170</v>
+        <v>25</v>
       </c>
       <c r="M15" s="2" t="s">
         <v>171</v>
@@ -1871,25 +1907,23 @@
         <v>173</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>41</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E16" s="2" t="s">
         <v>177</v>
       </c>
+      <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
         <v>20</v>
       </c>
@@ -1909,47 +1943,51 @@
         <v>1</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>25</v>
+        <v>182</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="P16" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>189</v>
+        <v>20</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
+      <c r="H17" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>192</v>
+      </c>
       <c r="J17" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="K17" s="2" t="n">
         <v>1</v>
@@ -1958,186 +1996,232 @@
         <v>25</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="G18" s="2"/>
+        <v>201</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>202</v>
+      </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="K18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>83</v>
+        <v>25</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="O18" s="2"/>
+        <v>205</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>206</v>
+      </c>
       <c r="P18" s="2" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C19" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>209</v>
-      </c>
+        <v>212</v>
+      </c>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>211</v>
+        <v>95</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="O19" s="2" t="s">
-        <v>214</v>
-      </c>
+        <v>215</v>
+      </c>
+      <c r="O19" s="2"/>
       <c r="P19" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C20" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="E20" s="2"/>
+        <v>219</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>220</v>
+      </c>
       <c r="F20" s="2" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="H20" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>221</v>
+      </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="O20" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="P20" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="P20" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="B22" s="4" t="n">
-        <f aca="false">COUNTA(A2:A20)</f>
-        <v>19</v>
+      <c r="M21" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="O21" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="P21" s="2" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
       <c r="B23" s="4" t="n">
-        <f aca="false">SUM(K2:K20)</f>
-        <v>41</v>
+        <f aca="false">COUNTA(A2:A21)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="B24" s="4" t="n">
-        <f aca="false">COUNTIF(N2:N20,"*.pdf")</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
-        <v>228</v>
+        <f aca="false">SUM(K2:K21)</f>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="B25" s="4" t="n">
+        <f aca="false">COUNTIF(N2:N21,"*.pdf")</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>240</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P20"/>
+  <autoFilter ref="A1:P21"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>